<commit_message>
QTL Quan Ly Ho So UF
</commit_message>
<xml_diff>
--- a/Quan Trac Lun/Data/HD XL01/KM0+400.xlsx
+++ b/Quan Trac Lun/Data/HD XL01/KM0+400.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vba\bketech\Quan Trac Lun\Data\HD XL01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E142E46F-3C40-4E4D-B4FA-5DE7FD85227C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2507415-B49C-4880-9045-7F316988FB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{2C402617-1403-418F-9928-C6EF4DD57BF2}"/>
+    <workbookView xWindow="-8325" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{2C402617-1403-418F-9928-C6EF4DD57BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -552,16 +552,25 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -616,15 +625,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -975,139 +975,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="32.450000000000003" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27"/>
-      <c r="V1" s="27"/>
-      <c r="W1" s="27"/>
-      <c r="X1" s="27"/>
-      <c r="Y1" s="27"/>
-      <c r="Z1" s="27"/>
-      <c r="AA1" s="27"/>
-      <c r="AB1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="30"/>
+      <c r="T1" s="30"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
+      <c r="W1" s="30"/>
+      <c r="X1" s="30"/>
+      <c r="Y1" s="30"/>
+      <c r="Z1" s="30"/>
+      <c r="AA1" s="30"/>
+      <c r="AB1" s="31"/>
     </row>
     <row r="2" spans="1:28" ht="17.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="30"/>
-      <c r="V2" s="30"/>
-      <c r="W2" s="30"/>
-      <c r="X2" s="30"/>
-      <c r="Y2" s="30"/>
-      <c r="Z2" s="30"/>
-      <c r="AA2" s="30"/>
-      <c r="AB2" s="31"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="33"/>
+      <c r="R2" s="33"/>
+      <c r="S2" s="33"/>
+      <c r="T2" s="33"/>
+      <c r="U2" s="33"/>
+      <c r="V2" s="33"/>
+      <c r="W2" s="33"/>
+      <c r="X2" s="33"/>
+      <c r="Y2" s="33"/>
+      <c r="Z2" s="33"/>
+      <c r="AA2" s="33"/>
+      <c r="AB2" s="34"/>
     </row>
     <row r="3" spans="1:28" ht="17.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="30"/>
-      <c r="R3" s="30"/>
-      <c r="S3" s="30"/>
-      <c r="T3" s="30"/>
-      <c r="U3" s="30"/>
-      <c r="V3" s="30"/>
-      <c r="W3" s="30"/>
-      <c r="X3" s="30"/>
-      <c r="Y3" s="30"/>
-      <c r="Z3" s="30"/>
-      <c r="AA3" s="30"/>
-      <c r="AB3" s="31"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="33"/>
+      <c r="O3" s="33"/>
+      <c r="P3" s="33"/>
+      <c r="Q3" s="33"/>
+      <c r="R3" s="33"/>
+      <c r="S3" s="33"/>
+      <c r="T3" s="33"/>
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
+      <c r="Y3" s="33"/>
+      <c r="Z3" s="33"/>
+      <c r="AA3" s="33"/>
+      <c r="AB3" s="34"/>
     </row>
     <row r="4" spans="1:28" ht="17.25">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
-      <c r="Q4" s="33"/>
-      <c r="R4" s="33"/>
-      <c r="S4" s="33"/>
-      <c r="T4" s="33"/>
-      <c r="U4" s="33"/>
-      <c r="V4" s="33"/>
-      <c r="W4" s="33"/>
-      <c r="X4" s="33"/>
-      <c r="Y4" s="33"/>
-      <c r="Z4" s="33"/>
-      <c r="AA4" s="33"/>
-      <c r="AB4" s="34"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="36"/>
+      <c r="S4" s="36"/>
+      <c r="T4" s="36"/>
+      <c r="U4" s="36"/>
+      <c r="V4" s="36"/>
+      <c r="W4" s="36"/>
+      <c r="X4" s="36"/>
+      <c r="Y4" s="36"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="36"/>
+      <c r="AB4" s="37"/>
     </row>
     <row r="5" spans="1:28">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -1137,11 +1137,11 @@
       <c r="AB5" s="4"/>
     </row>
     <row r="6" spans="1:28">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="41"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -1173,13 +1173,13 @@
       <c r="AB6" s="9"/>
     </row>
     <row r="7" spans="1:28">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="40"/>
+      <c r="C7" s="43"/>
       <c r="D7" s="10" t="s">
         <v>34</v>
       </c>
@@ -1213,71 +1213,71 @@
       <c r="AB7" s="13"/>
     </row>
     <row r="8" spans="1:28" ht="13.9" customHeight="1">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="21"/>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="23" t="s">
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="J8" s="24"/>
-      <c r="K8" s="24"/>
-      <c r="L8" s="23" t="s">
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="M8" s="24"/>
-      <c r="N8" s="25"/>
-      <c r="O8" s="23" t="s">
+      <c r="M8" s="23"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="P8" s="24"/>
-      <c r="Q8" s="25"/>
-      <c r="R8" s="44" t="s">
+      <c r="P8" s="23"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="S8" s="46"/>
-      <c r="T8" s="45"/>
-      <c r="U8" s="44" t="s">
+      <c r="S8" s="26"/>
+      <c r="T8" s="27"/>
+      <c r="U8" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="V8" s="46"/>
-      <c r="W8" s="45"/>
-      <c r="X8" s="22" t="s">
+      <c r="V8" s="26"/>
+      <c r="W8" s="27"/>
+      <c r="X8" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="Y8" s="22" t="s">
+      <c r="Y8" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="Z8" s="22" t="s">
+      <c r="Z8" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="AA8" s="44" t="s">
+      <c r="AA8" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="AB8" s="45"/>
+      <c r="AB8" s="27"/>
     </row>
     <row r="9" spans="1:28" ht="30">
-      <c r="A9" s="42"/>
+      <c r="A9" s="45"/>
       <c r="B9" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="22"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="28"/>
       <c r="F9" s="14" t="s">
         <v>22</v>
       </c>
@@ -1332,9 +1332,9 @@
       <c r="W9" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="X9" s="22"/>
-      <c r="Y9" s="22"/>
-      <c r="Z9" s="22"/>
+      <c r="X9" s="28"/>
+      <c r="Y9" s="28"/>
+      <c r="Z9" s="28"/>
       <c r="AA9" s="14" t="s">
         <v>25</v>
       </c>
@@ -1343,54 +1343,54 @@
       </c>
     </row>
     <row r="10" spans="1:28" ht="30">
-      <c r="A10" s="43"/>
+      <c r="A10" s="46"/>
       <c r="B10" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q10" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R10" s="18" t="s">
         <v>28</v>
@@ -1504,11 +1504,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="O8:Q8"/>
-    <mergeCell ref="R8:T8"/>
-    <mergeCell ref="U8:W8"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="Y8:Y9"/>
     <mergeCell ref="E8:E9"/>
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="I8:K8"/>
@@ -1525,6 +1520,11 @@
     <mergeCell ref="D8:D9"/>
     <mergeCell ref="AA8:AB8"/>
     <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="O8:Q8"/>
+    <mergeCell ref="R8:T8"/>
+    <mergeCell ref="U8:W8"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="Y8:Y9"/>
   </mergeCells>
   <pageMargins left="0.19685039370078741" right="7.874015748031496E-2" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>